<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-15 21:55:00
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-24 16:01:51
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-30 22:54:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-17 17:50:47
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-18 14:00:35
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-20 23:01:56
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-21 15:49:12
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-21 17:23:32
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-23 16:24:15
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-24 16:13:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-24 18:47:40
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-24 20:43:45
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-24 22:11:42
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-25 04:59:44
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-26 10:18:50
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-27 23:04:17
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-28 16:05:51
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-01 00:02:39
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-05 11:26:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-05 17:02:27
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-05 19:07:32
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-05 20:51:54
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-06 21:24:11
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-06 23:01:59
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-08 17:23:57
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-10 13:07:43
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-10 20:17:48
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-10 21:56:04
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 05:51:11
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 13:06:01
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-12 14:50:42
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-14 17:07:44
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-15 01:52:17
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-15 13:23:20
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-16 05:34:05
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-18 04:44:33
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-21 02:05:16
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-22 05:43:09
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-23 08:20:38
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-26 14:59:43
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-29 02:39:35
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-07-29 22:55:55
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-01 10:35:43
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-01 13:23:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-01 14:55:07
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-03 13:35:40
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-03 22:02:27
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-04 00:03:03
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-05 17:38:32
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-07 11:40:34
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-08 06:40:30
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-09 10:27:15
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-09 19:27:55
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-10 20:35:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-11 06:56:21
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-11 17:53:30
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-12 11:42:14
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2526, 2025/2026</t>
+          <t>2025/2026, 2526</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-13 06:11:45
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-13 09:57:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-08-13 17:52:46
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A2_session_analysis.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -12543,7 +12543,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -15053,7 +15053,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2526</t>
+          <t>2526, 2025/2026</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">

</xml_diff>